<commit_message>
Infer leaders for TRGs without a labeled leader; KPI shows TRGs with a leader
247 of 277 TRGs now have a leader (231 labeled on site + 16 inferred, listed in ketua_diduga.csv).
KPI counts TRGs, not people.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VuHePFv7oto5SNMHb2pbjZ
</commit_message>
<xml_diff>
--- a/forms/trg/Formulir_TRG_aisrg.xlsx
+++ b/forms/trg/Formulir_TRG_aisrg.xlsx
@@ -916,7 +916,11 @@
           <t>Prof. Dr. Ir. Sitti Bulkis, M.S.</t>
         </is>
       </c>
-      <c r="C5" s="12" t="n"/>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Leader</t>
+        </is>
+      </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
           <t>Agricultural Institutions, Gender, and Food Security</t>

</xml_diff>